<commit_message>
solved initial load app of the app
</commit_message>
<xml_diff>
--- a/data/C GST.xlsx
+++ b/data/C GST.xlsx
@@ -581,7 +581,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="72">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -860,14 +860,6 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -901,9 +893,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>266400</xdr:colOff>
+      <xdr:colOff>266040</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>149760</xdr:rowOff>
+      <xdr:rowOff>149400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -916,47 +908,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9719280" y="9410760"/>
-          <a:ext cx="9360" cy="9360"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>235440</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1066680</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>578160</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 4" descr=""/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10795680" y="12744360"/>
-          <a:ext cx="1841400" cy="590400"/>
+          <a:off x="9718560" y="9410760"/>
+          <a:ext cx="9000" cy="9000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1661,11 +1614,11 @@
       <c r="H47" s="46"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="70" t="s">
+      <c r="A48" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B48" s="71"/>
-      <c r="C48" s="71"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
@@ -1692,23 +1645,23 @@
       <c r="C50" s="64"/>
       <c r="D50" s="64"/>
       <c r="E50" s="64"/>
-      <c r="F50" s="72" t="s">
+      <c r="F50" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="G50" s="72"/>
-      <c r="H50" s="72"/>
+      <c r="G50" s="70"/>
+      <c r="H50" s="70"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="73" t="s">
+      <c r="A51" s="71" t="s">
         <v>56</v>
       </c>
-      <c r="B51" s="73"/>
-      <c r="C51" s="73"/>
-      <c r="D51" s="73"/>
-      <c r="E51" s="73"/>
-      <c r="F51" s="73"/>
-      <c r="G51" s="73"/>
-      <c r="H51" s="73"/>
+      <c r="B51" s="71"/>
+      <c r="C51" s="71"/>
+      <c r="D51" s="71"/>
+      <c r="E51" s="71"/>
+      <c r="F51" s="71"/>
+      <c r="G51" s="71"/>
+      <c r="H51" s="71"/>
     </row>
     <row r="52" customFormat="false" ht="0.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>